<commit_message>
Lot 4 : Petritsi, Milarépa, Gampopa, Gökalp, Topçu, Næss, von Wright, Hintikka, Marković, Petrović, Kuçuradi ; Géorgie dans Grecs & Byzantins ; slug : lettres liées (æ, œ, ø…) converties
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-medievaux.xlsx
+++ b/data/frise-philosophes-medievaux.xlsx
@@ -598,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N115"/>
+  <dimension ref="A1:P116"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6.81" customWidth="1" style="23" min="1" max="1"/>
@@ -8263,7 +8263,64 @@
         </is>
       </c>
     </row>
-    <row r="116" ht="76.5" customHeight="1" s="25"/>
+    <row r="116" ht="76.5" customHeight="1" s="25">
+      <c r="A116" s="30">
+        <v>1060</v>
+      </c>
+      <c r="B116" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1130</t>
+        </is>
+      </c>
+      <c r="C116" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XIe – XIIe siècle</t>
+        </is>
+      </c>
+      <c r="D116" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ioane PETRITSI</t>
+        </is>
+      </c>
+      <c r="E116" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Ioane_Petritsi" title=" Wikipedia (en)"&gt;Ioane PETRITSI&lt;/a&gt; est le plus important philosophe géorgien du Moyen Âge. Né dans une famille aristocratique de la province de Samtskhé, dans le sud de la Géorgie, il étudie à Constantinople auprès des plus grands maîtres byzantins de son temps, Michel Psellos et Jean Italos, qui renouvellent l’étude de Platon et des néoplatoniciens. Après la condamnation de Jean Italos pour hérésie, il se réfugie, semble-t-il, au monastère géorgien de Petritsoni, en Bulgarie, dont il tire son surnom.&lt;/p&gt; &lt;p&gt;Traducteur infatigable, il fait passer en géorgien des œuvres d’Aristote, de &lt;a href="https://fr.wikipedia.org/wiki/Proclus" title=" Wikipedia"&gt;Proclus&lt;/a&gt;, de Némésius et d’Ammonius, ainsi que des textes bibliques et des vies de saints. Il veut montrer que la philosophie grecque et la foi chrétienne peuvent s’accorder. Son œuvre maîtresse est sa traduction des &lt;em&gt;Éléments de théologie&lt;/em&gt; de Proclus, accompagnée d’un long commentaire : l’Un, principe premier au-delà de tout ce qui existe, y est rapproché du Dieu chrétien, et la procession des êtres à partir de l’Un est relue à la lumière de la Création.&lt;/p&gt; &lt;p&gt;Ses idées le mettent en conflit avec les gardiens de l’orthodoxie géorgienne, jusqu’à ce que le roi David IV le Bâtisseur l’installe à l’académie de Gelati, grand centre d’enseignement fondé par le souverain. Il compose aussi des hymnes et de la poésie mystique. Son influence sur la pensée et la langue philosophique géorgiennes a été durable, et elle connaît un renouveau au XVIIIe siècle. Il est aujourd’hui considéré comme le philosophe géorgien le plus lu.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H116" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/petritsi-mini.webp</t>
+        </is>
+      </c>
+      <c r="J116" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Géorgienne</t>
+        </is>
+      </c>
+      <c r="K116" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique ; spiritualite</t>
+        </is>
+      </c>
+      <c r="L116" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Néoplatonisme</t>
+        </is>
+      </c>
+      <c r="M116" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophe néoplatonicien géorgien, traducteur et commentateur de Proclus.</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="P116">
+        <v>2</v>
+      </c>
+    </row>
     <row r="117" ht="99.75" customHeight="1" s="25"/>
   </sheetData>
   <mergeCells count="2">

</xml_diff>